<commit_message>
chero update's from figures around
</commit_message>
<xml_diff>
--- a/2026/outputs/TOR_A_long_table_bycatch_only.xlsx
+++ b/2026/outputs/TOR_A_long_table_bycatch_only.xlsx
@@ -9289,7 +9289,7 @@
         <v>16</v>
       </c>
       <c r="D234" t="n">
-        <v>474.116666666666</v>
+        <v>474.116666666667</v>
       </c>
       <c r="E234" t="s">
         <v>34</v>
@@ -9324,7 +9324,7 @@
         <v>16</v>
       </c>
       <c r="D235" t="n">
-        <v>474.116666666666</v>
+        <v>474.116666666667</v>
       </c>
       <c r="E235" t="s">
         <v>14</v>
@@ -11115,7 +11115,7 @@
         <v>81</v>
       </c>
       <c r="F286" t="n">
-        <v>3506.39328388402</v>
+        <v>3506.39328388403</v>
       </c>
       <c r="G286" t="n">
         <v>10.6865340311869</v>
@@ -11150,7 +11150,7 @@
         <v>81</v>
       </c>
       <c r="F287" t="n">
-        <v>3506.39328388402</v>
+        <v>3506.39328388403</v>
       </c>
       <c r="G287" t="n">
         <v>10.6865340311869</v>
@@ -11185,7 +11185,7 @@
         <v>81</v>
       </c>
       <c r="F288" t="n">
-        <v>3506.39328388402</v>
+        <v>3506.39328388403</v>
       </c>
       <c r="G288" t="n">
         <v>10.6865340311869</v>
@@ -11564,7 +11564,7 @@
         <v>39</v>
       </c>
       <c r="D299" t="n">
-        <v>3357.31630306152</v>
+        <v>3357.31630306153</v>
       </c>
       <c r="E299" t="s">
         <v>14</v>
@@ -11599,7 +11599,7 @@
         <v>39</v>
       </c>
       <c r="D300" t="n">
-        <v>3357.31630306152</v>
+        <v>3357.31630306153</v>
       </c>
       <c r="E300" t="s">
         <v>14</v>
@@ -14336,7 +14336,7 @@
         <v>422</v>
       </c>
       <c r="G378" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H378" t="s">
         <v>30</v>
@@ -14371,7 +14371,7 @@
         <v>422</v>
       </c>
       <c r="G379" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H379" t="s">
         <v>30</v>
@@ -14406,7 +14406,7 @@
         <v>422</v>
       </c>
       <c r="G380" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H380" t="s">
         <v>30</v>
@@ -14441,7 +14441,7 @@
         <v>422</v>
       </c>
       <c r="G381" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H381" t="s">
         <v>18</v>
@@ -14476,7 +14476,7 @@
         <v>422</v>
       </c>
       <c r="G382" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H382" t="s">
         <v>61</v>
@@ -14511,7 +14511,7 @@
         <v>422</v>
       </c>
       <c r="G383" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H383" t="s">
         <v>30</v>
@@ -14546,7 +14546,7 @@
         <v>422</v>
       </c>
       <c r="G384" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H384" t="s">
         <v>18</v>
@@ -14581,7 +14581,7 @@
         <v>422</v>
       </c>
       <c r="G385" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H385" t="s">
         <v>42</v>
@@ -14616,7 +14616,7 @@
         <v>422</v>
       </c>
       <c r="G386" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H386" t="s">
         <v>18</v>
@@ -14651,7 +14651,7 @@
         <v>422</v>
       </c>
       <c r="G387" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H387" t="s">
         <v>30</v>
@@ -14686,7 +14686,7 @@
         <v>422</v>
       </c>
       <c r="G388" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H388" t="s">
         <v>18</v>
@@ -14721,7 +14721,7 @@
         <v>422</v>
       </c>
       <c r="G389" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H389" t="s">
         <v>18</v>
@@ -14756,7 +14756,7 @@
         <v>422</v>
       </c>
       <c r="G390" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H390" t="s">
         <v>30</v>
@@ -14791,7 +14791,7 @@
         <v>422</v>
       </c>
       <c r="G391" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H391" t="s">
         <v>18</v>
@@ -14826,7 +14826,7 @@
         <v>422</v>
       </c>
       <c r="G392" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H392" t="s">
         <v>30</v>
@@ -14861,7 +14861,7 @@
         <v>422</v>
       </c>
       <c r="G393" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H393" t="s">
         <v>30</v>
@@ -14896,7 +14896,7 @@
         <v>422</v>
       </c>
       <c r="G394" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H394" t="s">
         <v>30</v>
@@ -14931,7 +14931,7 @@
         <v>422</v>
       </c>
       <c r="G395" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H395" t="s">
         <v>30</v>
@@ -14966,7 +14966,7 @@
         <v>422</v>
       </c>
       <c r="G396" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H396" t="s">
         <v>30</v>
@@ -15001,7 +15001,7 @@
         <v>422</v>
       </c>
       <c r="G397" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H397" t="s">
         <v>18</v>
@@ -15036,7 +15036,7 @@
         <v>422</v>
       </c>
       <c r="G398" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H398" t="s">
         <v>18</v>
@@ -15071,7 +15071,7 @@
         <v>422</v>
       </c>
       <c r="G399" t="n">
-        <v>2.9935097947945</v>
+        <v>2.99350979479449</v>
       </c>
       <c r="H399" t="s">
         <v>30</v>
@@ -17652,7 +17652,7 @@
         <v>39</v>
       </c>
       <c r="D473" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E473" t="s">
         <v>14</v>
@@ -17661,7 +17661,7 @@
         <v>108.83</v>
       </c>
       <c r="G473" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H473" t="s">
         <v>30</v>
@@ -17687,7 +17687,7 @@
         <v>39</v>
       </c>
       <c r="D474" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E474" t="s">
         <v>14</v>
@@ -17696,7 +17696,7 @@
         <v>108.83</v>
       </c>
       <c r="G474" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H474" t="s">
         <v>30</v>
@@ -17722,7 +17722,7 @@
         <v>39</v>
       </c>
       <c r="D475" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E475" t="s">
         <v>14</v>
@@ -17731,7 +17731,7 @@
         <v>108.83</v>
       </c>
       <c r="G475" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H475" t="s">
         <v>30</v>
@@ -17757,7 +17757,7 @@
         <v>39</v>
       </c>
       <c r="D476" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E476" t="s">
         <v>14</v>
@@ -17766,7 +17766,7 @@
         <v>108.83</v>
       </c>
       <c r="G476" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H476" t="s">
         <v>18</v>
@@ -17792,7 +17792,7 @@
         <v>39</v>
       </c>
       <c r="D477" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E477" t="s">
         <v>14</v>
@@ -17801,7 +17801,7 @@
         <v>108.83</v>
       </c>
       <c r="G477" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H477" t="s">
         <v>18</v>
@@ -17827,7 +17827,7 @@
         <v>39</v>
       </c>
       <c r="D478" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E478" t="s">
         <v>14</v>
@@ -17836,7 +17836,7 @@
         <v>108.83</v>
       </c>
       <c r="G478" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H478" t="s">
         <v>61</v>
@@ -17862,7 +17862,7 @@
         <v>39</v>
       </c>
       <c r="D479" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E479" t="s">
         <v>14</v>
@@ -17871,7 +17871,7 @@
         <v>108.83</v>
       </c>
       <c r="G479" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H479" t="s">
         <v>30</v>
@@ -17897,7 +17897,7 @@
         <v>39</v>
       </c>
       <c r="D480" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E480" t="s">
         <v>14</v>
@@ -17906,7 +17906,7 @@
         <v>108.83</v>
       </c>
       <c r="G480" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H480" t="s">
         <v>30</v>
@@ -17932,7 +17932,7 @@
         <v>39</v>
       </c>
       <c r="D481" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E481" t="s">
         <v>14</v>
@@ -17941,7 +17941,7 @@
         <v>108.83</v>
       </c>
       <c r="G481" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H481" t="s">
         <v>18</v>
@@ -17967,7 +17967,7 @@
         <v>39</v>
       </c>
       <c r="D482" t="n">
-        <v>2466.10108614181</v>
+        <v>2466.1010861418</v>
       </c>
       <c r="E482" t="s">
         <v>14</v>
@@ -17976,7 +17976,7 @@
         <v>108.83</v>
       </c>
       <c r="G482" t="n">
-        <v>4.413038890075</v>
+        <v>4.41303889007501</v>
       </c>
       <c r="H482" t="s">
         <v>18</v>
@@ -19061,7 +19061,7 @@
         <v>28.12</v>
       </c>
       <c r="G513" t="n">
-        <v>9.7674930273679</v>
+        <v>9.76749302736789</v>
       </c>
       <c r="H513" t="s">
         <v>30</v>
@@ -19096,7 +19096,7 @@
         <v>28.12</v>
       </c>
       <c r="G514" t="n">
-        <v>9.7674930273679</v>
+        <v>9.76749302736789</v>
       </c>
       <c r="H514" t="s">
         <v>18</v>
@@ -19131,7 +19131,7 @@
         <v>28.12</v>
       </c>
       <c r="G515" t="n">
-        <v>9.7674930273679</v>
+        <v>9.76749302736789</v>
       </c>
       <c r="H515" t="s">
         <v>18</v>
@@ -19166,7 +19166,7 @@
         <v>28.12</v>
       </c>
       <c r="G516" t="n">
-        <v>9.7674930273679</v>
+        <v>9.76749302736789</v>
       </c>
       <c r="H516" t="s">
         <v>18</v>
@@ -20531,7 +20531,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G555" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H555" t="s">
         <v>30</v>
@@ -20566,7 +20566,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G556" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H556" t="s">
         <v>18</v>
@@ -20601,7 +20601,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G557" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H557" t="s">
         <v>18</v>
@@ -20636,7 +20636,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G558" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H558" t="s">
         <v>18</v>
@@ -20671,7 +20671,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G559" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H559" t="s">
         <v>18</v>
@@ -20706,7 +20706,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G560" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H560" t="s">
         <v>18</v>
@@ -20741,7 +20741,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G561" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H561" t="s">
         <v>18</v>
@@ -20776,7 +20776,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G562" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H562" t="s">
         <v>30</v>
@@ -20811,7 +20811,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G563" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H563" t="s">
         <v>30</v>
@@ -20846,7 +20846,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G564" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H564" t="s">
         <v>18</v>
@@ -20881,7 +20881,7 @@
         <v>42.757575758</v>
       </c>
       <c r="G565" t="n">
-        <v>2.79848098199146</v>
+        <v>2.79848098199147</v>
       </c>
       <c r="H565" t="s">
         <v>30</v>
@@ -21439,7 +21439,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G581" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H581" t="s">
         <v>18</v>
@@ -21474,7 +21474,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G582" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H582" t="s">
         <v>18</v>
@@ -21509,7 +21509,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G583" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H583" t="s">
         <v>18</v>
@@ -21544,7 +21544,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G584" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H584" t="s">
         <v>25</v>
@@ -21579,7 +21579,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G585" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H585" t="s">
         <v>42</v>
@@ -21614,7 +21614,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G586" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H586" t="s">
         <v>18</v>
@@ -21649,7 +21649,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G587" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H587" t="s">
         <v>30</v>
@@ -21684,7 +21684,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G588" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H588" t="s">
         <v>18</v>
@@ -21719,7 +21719,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G589" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H589" t="s">
         <v>18</v>
@@ -21754,7 +21754,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G590" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H590" t="s">
         <v>18</v>
@@ -21789,7 +21789,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G591" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H591" t="s">
         <v>30</v>
@@ -21824,7 +21824,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G592" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H592" t="s">
         <v>30</v>
@@ -21859,7 +21859,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G593" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H593" t="s">
         <v>30</v>
@@ -21894,7 +21894,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G594" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H594" t="s">
         <v>18</v>
@@ -21929,7 +21929,7 @@
         <v>59.906656347</v>
       </c>
       <c r="G595" t="n">
-        <v>1.50954485063963</v>
+        <v>1.50954485063962</v>
       </c>
       <c r="H595" t="s">
         <v>30</v>
@@ -27284,7 +27284,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G748" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H748" t="s">
         <v>30</v>
@@ -27319,7 +27319,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G749" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H749" t="s">
         <v>18</v>
@@ -27354,7 +27354,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G750" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H750" t="s">
         <v>30</v>
@@ -27389,7 +27389,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G751" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H751" t="s">
         <v>61</v>
@@ -27424,7 +27424,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G752" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H752" t="s">
         <v>18</v>
@@ -27459,7 +27459,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G753" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H753" t="s">
         <v>18</v>
@@ -27494,7 +27494,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G754" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H754" t="s">
         <v>30</v>
@@ -27529,7 +27529,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G755" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H755" t="s">
         <v>30</v>
@@ -27564,7 +27564,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G756" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H756" t="s">
         <v>18</v>
@@ -27599,7 +27599,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G757" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H757" t="s">
         <v>18</v>
@@ -27634,7 +27634,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G758" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H758" t="s">
         <v>30</v>
@@ -27669,7 +27669,7 @@
         <v>205.723333333333</v>
       </c>
       <c r="G759" t="n">
-        <v>0.481051646739637</v>
+        <v>0.481051646739636</v>
       </c>
       <c r="H759" t="s">
         <v>30</v>
@@ -28080,7 +28080,7 @@
         <v>44</v>
       </c>
       <c r="D771" t="n">
-        <v>18370.1453132334</v>
+        <v>18370.1453132333</v>
       </c>
       <c r="E771" t="s">
         <v>14</v>
@@ -28089,7 +28089,7 @@
         <v>141.86246031746</v>
       </c>
       <c r="G771" t="n">
-        <v>0.772244627892336</v>
+        <v>0.772244627892337</v>
       </c>
       <c r="H771" t="s">
         <v>30</v>
@@ -28115,7 +28115,7 @@
         <v>44</v>
       </c>
       <c r="D772" t="n">
-        <v>18370.1453132334</v>
+        <v>18370.1453132333</v>
       </c>
       <c r="E772" t="s">
         <v>14</v>
@@ -28124,7 +28124,7 @@
         <v>141.86246031746</v>
       </c>
       <c r="G772" t="n">
-        <v>0.772244627892336</v>
+        <v>0.772244627892337</v>
       </c>
       <c r="H772" t="s">
         <v>18</v>
@@ -28150,7 +28150,7 @@
         <v>44</v>
       </c>
       <c r="D773" t="n">
-        <v>18370.1453132334</v>
+        <v>18370.1453132333</v>
       </c>
       <c r="E773" t="s">
         <v>14</v>
@@ -28159,7 +28159,7 @@
         <v>141.86246031746</v>
       </c>
       <c r="G773" t="n">
-        <v>0.772244627892336</v>
+        <v>0.772244627892337</v>
       </c>
       <c r="H773" t="s">
         <v>18</v>
@@ -28185,7 +28185,7 @@
         <v>44</v>
       </c>
       <c r="D774" t="n">
-        <v>18370.1453132334</v>
+        <v>18370.1453132333</v>
       </c>
       <c r="E774" t="s">
         <v>14</v>
@@ -28194,7 +28194,7 @@
         <v>141.86246031746</v>
       </c>
       <c r="G774" t="n">
-        <v>0.772244627892336</v>
+        <v>0.772244627892337</v>
       </c>
       <c r="H774" t="s">
         <v>18</v>
@@ -28220,7 +28220,7 @@
         <v>44</v>
       </c>
       <c r="D775" t="n">
-        <v>18370.1453132334</v>
+        <v>18370.1453132333</v>
       </c>
       <c r="E775" t="s">
         <v>14</v>
@@ -28229,7 +28229,7 @@
         <v>141.86246031746</v>
       </c>
       <c r="G775" t="n">
-        <v>0.772244627892336</v>
+        <v>0.772244627892337</v>
       </c>
       <c r="H775" t="s">
         <v>30</v>
@@ -28264,7 +28264,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G776" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H776" t="s">
         <v>102</v>
@@ -28299,7 +28299,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G777" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H777" t="s">
         <v>25</v>
@@ -28334,7 +28334,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G778" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H778" t="s">
         <v>42</v>
@@ -28369,7 +28369,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G779" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H779" t="s">
         <v>42</v>
@@ -28404,7 +28404,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G780" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H780" t="s">
         <v>18</v>
@@ -28439,7 +28439,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G781" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H781" t="s">
         <v>18</v>
@@ -28474,7 +28474,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G782" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H782" t="s">
         <v>18</v>
@@ -28509,7 +28509,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G783" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H783" t="s">
         <v>42</v>
@@ -28544,7 +28544,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G784" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H784" t="s">
         <v>18</v>
@@ -28579,7 +28579,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G785" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H785" t="s">
         <v>25</v>
@@ -28614,7 +28614,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G786" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H786" t="s">
         <v>42</v>
@@ -28649,7 +28649,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G787" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H787" t="s">
         <v>42</v>
@@ -28684,7 +28684,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G788" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H788" t="s">
         <v>18</v>
@@ -28719,7 +28719,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G789" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H789" t="s">
         <v>18</v>
@@ -28754,7 +28754,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G790" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H790" t="s">
         <v>18</v>
@@ -28789,7 +28789,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G791" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H791" t="s">
         <v>18</v>
@@ -28824,7 +28824,7 @@
         <v>396.915068761905</v>
       </c>
       <c r="G792" t="n">
-        <v>3.07820823032026</v>
+        <v>3.07820823032025</v>
       </c>
       <c r="H792" t="s">
         <v>25</v>
@@ -28859,7 +28859,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G793" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H793" t="s">
         <v>25</v>
@@ -28894,7 +28894,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G794" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H794" t="s">
         <v>18</v>
@@ -28929,7 +28929,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G795" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H795" t="s">
         <v>42</v>
@@ -28964,7 +28964,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G796" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H796" t="s">
         <v>18</v>
@@ -28999,7 +28999,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G797" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H797" t="s">
         <v>18</v>
@@ -29034,7 +29034,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G798" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H798" t="s">
         <v>25</v>
@@ -29069,7 +29069,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G799" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H799" t="s">
         <v>42</v>
@@ -29104,7 +29104,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G800" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H800" t="s">
         <v>18</v>
@@ -29139,7 +29139,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G801" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H801" t="s">
         <v>18</v>
@@ -29174,7 +29174,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G802" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H802" t="s">
         <v>30</v>
@@ -29209,7 +29209,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G803" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H803" t="s">
         <v>25</v>
@@ -29244,7 +29244,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G804" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H804" t="s">
         <v>42</v>
@@ -29279,7 +29279,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G805" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H805" t="s">
         <v>30</v>
@@ -29314,7 +29314,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G806" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H806" t="s">
         <v>18</v>
@@ -29349,7 +29349,7 @@
         <v>122.472622152278</v>
       </c>
       <c r="G807" t="n">
-        <v>0.949815875406316</v>
+        <v>0.949815875406315</v>
       </c>
       <c r="H807" t="s">
         <v>30</v>
@@ -29384,7 +29384,7 @@
         <v>5.05636363636364</v>
       </c>
       <c r="G808" t="n">
-        <v>0.825121721111817</v>
+        <v>0.825121721111818</v>
       </c>
       <c r="H808" t="s">
         <v>25</v>

</xml_diff>